<commit_message>
nueva galeria e imagenes
</commit_message>
<xml_diff>
--- a/eventos-plantilla.xlsx
+++ b/eventos-plantilla.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="167">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -170,7 +170,7 @@
     <t xml:space="preserve">103-a.C.</t>
   </si>
   <si>
-    <t xml:space="preserve">Poder y Corrupción</t>
+    <t xml:space="preserve">Personajes históricos</t>
   </si>
   <si>
     <t xml:space="preserve">/images/eventos/Roma-juicios-por-traición.jpg</t>
@@ -256,9 +256,6 @@
   </si>
   <si>
     <t xml:space="preserve">Cuauhtémoc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Personajes históricos</t>
   </si>
   <si>
     <t xml:space="preserve">/images/eventos/Cuauhtemoc.jpg</t>
@@ -992,7 +989,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1021,6 +1018,12 @@
       <name val="Aptos Narrow"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1065,7 +1068,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1083,6 +1086,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1350,7 +1357,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="60.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="7" style="1" width="80.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="27.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="84.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="84.94"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1387,7 +1394,7 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1425,7 +1432,7 @@
       <c r="K2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="L2" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1474,7 +1481,7 @@
       <c r="C4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="5" t="s">
         <v>35</v>
       </c>
       <c r="E4" s="3" t="s">
@@ -1580,25 +1587,25 @@
         <v>1495</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="J7" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>62</v>
@@ -1606,150 +1613,150 @@
     </row>
     <row r="8" customFormat="false" ht="699" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="I8" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="J8" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="J8" s="5" t="s">
-        <v>80</v>
-      </c>
       <c r="K8" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="531" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>12512</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="I9" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="J9" s="3" t="s">
-        <v>88</v>
-      </c>
       <c r="K9" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="567" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="I10" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="J10" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="J10" s="3" t="s">
-        <v>98</v>
-      </c>
       <c r="K10" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="567" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="J11" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="K11" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="386.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>19958</v>
@@ -1758,103 +1765,103 @@
         <v>25</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="I12" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="J12" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="K12" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="326.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1840</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="I13" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="J13" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="J13" s="3" t="s">
-        <v>124</v>
-      </c>
       <c r="K13" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="615" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>1936</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="E14" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="I14" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="J14" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="J14" s="3" t="s">
-        <v>132</v>
-      </c>
       <c r="K14" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="362.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>1869</v>
@@ -1863,130 +1870,130 @@
         <v>25</v>
       </c>
       <c r="E15" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H15" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="I15" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="J15" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="J15" s="3" t="s">
-        <v>140</v>
-      </c>
       <c r="K15" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="326.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="I16" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="J16" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="J16" s="3" t="s">
-        <v>149</v>
-      </c>
       <c r="K16" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="D17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="H17" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="I17" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="J17" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="J17" s="3" t="s">
-        <v>158</v>
-      </c>
       <c r="K17" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="H18" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="I18" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="J18" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="J18" s="3" t="s">
-        <v>167</v>
-      </c>
       <c r="K18" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>